<commit_message>
Wed: 5-slide Rocco carousel + Benny I spy as 5th Meta post
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/campaigns/2026-10-07/POSTS.xlsx
+++ b/campaigns/2026-10-07/POSTS.xlsx
@@ -422,7 +422,7 @@
       <row>12</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1047750" cy="1314450"/>
+    <ext cx="1047750" cy="1866900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="9" name="Image 9" descr="Picture"/>
@@ -447,7 +447,7 @@
       <row>13</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1047750" cy="1866900"/>
+    <ext cx="1047750" cy="1314450"/>
     <pic>
       <nvPicPr>
         <cNvPr id="10" name="Image 10" descr="Picture"/>
@@ -572,7 +572,7 @@
       <row>18</row>
       <rowOff>0</rowOff>
     </from>
-    <ext cx="1047750" cy="1571625"/>
+    <ext cx="1047750" cy="1866900"/>
     <pic>
       <nvPicPr>
         <cNvPr id="15" name="Image 15" descr="Picture"/>
@@ -605,6 +605,31 @@
       </nvPicPr>
       <blipFill>
         <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId16"/>
+        <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
+          <a:fillRect/>
+        </a:stretch>
+      </blipFill>
+      <spPr>
+        <a:prstGeom xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" prst="rect"/>
+      </spPr>
+    </pic>
+    <clientData/>
+  </oneCellAnchor>
+  <oneCellAnchor>
+    <from>
+      <col>4</col>
+      <colOff>0</colOff>
+      <row>20</row>
+      <rowOff>0</rowOff>
+    </from>
+    <ext cx="1047750" cy="1571625"/>
+    <pic>
+      <nvPicPr>
+        <cNvPr id="17" name="Image 17" descr="Picture"/>
+        <cNvPicPr/>
+      </nvPicPr>
+      <blipFill>
+        <a:blip xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" cstate="print" r:embed="rId17"/>
         <a:stretch xmlns:a="http://schemas.openxmlformats.org/drawingml/2006/main">
           <a:fillRect/>
         </a:stretch>
@@ -907,7 +932,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J20"/>
+  <dimension ref="A1:J21"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="8" customWidth="1" min="1" max="1"/>
@@ -1122,121 +1147,163 @@
       </c>
     </row>
     <row r="8" ht="155" customHeight="1">
-      <c r="A8" s="4" t="inlineStr">
-        <is>
-          <t>✓</t>
-        </is>
-      </c>
-      <c r="B8" s="5" t="inlineStr">
+      <c r="A8" s="4" t="inlineStr"/>
+      <c r="B8" s="9" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C8" s="5" t="inlineStr">
-        <is>
-          <t>TikTok</t>
-        </is>
-      </c>
-      <c r="D8" s="5" t="inlineStr">
-        <is>
-          <t>Posy</t>
+      <c r="C8" s="9" t="inlineStr">
+        <is>
+          <t>Instagram + Facebook</t>
+        </is>
+      </c>
+      <c r="D8" s="9" t="inlineStr">
+        <is>
+          <t>Benny</t>
         </is>
       </c>
       <c r="E8" s="6" t="inlineStr"/>
       <c r="F8" s="7" t="inlineStr">
         <is>
-          <t>B-posy-color-quiz.mp4</t>
+          <t>E-benny-i-spy.mp4</t>
         </is>
       </c>
       <c r="G8" s="6" t="inlineStr"/>
       <c r="H8" s="6" t="inlineStr">
         <is>
+          <t>I spy, with my little eye... 🐻🦋 Can your toddler find it before I count to 3? Benny the Bear's Cozy Day is a coloring book kids color AND read. Ages 3-6.
+Get it on Amazon: https://www.amazon.com/dp/B0HLVSLXK7 (Instagram: link in bio)
+#ispy #toddleractivities #preschoolactivities #coloringbook</t>
+        </is>
+      </c>
+      <c r="I8" s="6" t="inlineStr">
+        <is>
+          <t>Did your toddler find Benny first? 🐻👇</t>
+        </is>
+      </c>
+      <c r="J8" s="6" t="inlineStr">
+        <is>
+          <t>Reel. Then share to Story with a link sticker.</t>
+        </is>
+      </c>
+    </row>
+    <row r="9" ht="155" customHeight="1">
+      <c r="A9" s="4" t="inlineStr">
+        <is>
+          <t>✓</t>
+        </is>
+      </c>
+      <c r="B9" s="5" t="inlineStr">
+        <is>
+          <t>18:30</t>
+        </is>
+      </c>
+      <c r="C9" s="5" t="inlineStr">
+        <is>
+          <t>TikTok</t>
+        </is>
+      </c>
+      <c r="D9" s="5" t="inlineStr">
+        <is>
+          <t>Posy</t>
+        </is>
+      </c>
+      <c r="E9" s="6" t="inlineStr"/>
+      <c r="F9" s="7" t="inlineStr">
+        <is>
+          <t>B-posy-color-quiz.mp4</t>
+        </is>
+      </c>
+      <c r="G9" s="6" t="inlineStr"/>
+      <c r="H9" s="6" t="inlineStr">
+        <is>
           <t>Color quiz for toddlers 🌈 Can your little one name all 3 before the timer? Unicorn coloring book that teaches colors AND reading. Ages 3-6. Link in bio
 #learncolors #toddlerlearning #unicorn #preschool #kidsquiz</t>
         </is>
       </c>
-      <c r="I8" s="6" t="inlineStr">
+      <c r="I9" s="6" t="inlineStr">
         <is>
           <t>How many did your kid get? 🌈👇</t>
         </is>
       </c>
-      <c r="J8" s="6" t="inlineStr">
+      <c r="J9" s="6" t="inlineStr">
         <is>
           <t>Already scheduled by Claude</t>
         </is>
       </c>
     </row>
-    <row r="9" ht="155" customHeight="1">
-      <c r="A9" s="4" t="inlineStr">
+    <row r="10" ht="155" customHeight="1">
+      <c r="A10" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B9" s="8" t="inlineStr">
+      <c r="B10" s="8" t="inlineStr">
         <is>
           <t>18:30</t>
         </is>
       </c>
-      <c r="C9" s="8" t="inlineStr">
+      <c r="C10" s="8" t="inlineStr">
         <is>
           <t>YouTube Shorts</t>
         </is>
       </c>
-      <c r="D9" s="8" t="inlineStr">
+      <c r="D10" s="8" t="inlineStr">
         <is>
           <t>Posy</t>
         </is>
       </c>
-      <c r="E9" s="6" t="inlineStr"/>
-      <c r="F9" s="7" t="inlineStr">
+      <c r="E10" s="6" t="inlineStr"/>
+      <c r="F10" s="7" t="inlineStr">
         <is>
           <t>B-posy-color-quiz.mp4</t>
         </is>
       </c>
-      <c r="G9" s="6" t="inlineStr">
+      <c r="G10" s="6" t="inlineStr">
         <is>
           <t>Color quiz for toddlers: can your kid name all 3? 🌈 #shorts</t>
         </is>
       </c>
-      <c r="H9" s="6" t="inlineStr">
+      <c r="H10" s="6" t="inlineStr">
         <is>
           <t>Learn colors with Posy the little unicorn! From "Posy the Little Unicorn's Rainbow Birthday", a color &amp; read book for kids 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLZF8NMX
 #learncolors #toddlerlearning #unicorn</t>
         </is>
       </c>
-      <c r="I9" s="6" t="inlineStr"/>
-      <c r="J9" s="6" t="inlineStr">
+      <c r="I10" s="6" t="inlineStr"/>
+      <c r="J10" s="6" t="inlineStr">
         <is>
           <t>Already scheduled by Claude (fix: set NOT made for kids)</t>
         </is>
       </c>
     </row>
-    <row r="10" ht="155" customHeight="1">
-      <c r="A10" s="4" t="inlineStr"/>
-      <c r="B10" s="9" t="inlineStr">
+    <row r="11" ht="155" customHeight="1">
+      <c r="A11" s="4" t="inlineStr"/>
+      <c r="B11" s="9" t="inlineStr">
         <is>
           <t>19:00</t>
         </is>
       </c>
-      <c r="C10" s="9" t="inlineStr">
+      <c r="C11" s="9" t="inlineStr">
         <is>
           <t>Instagram + Facebook</t>
         </is>
       </c>
-      <c r="D10" s="9" t="inlineStr">
+      <c r="D11" s="9" t="inlineStr">
         <is>
           <t>All 4</t>
         </is>
       </c>
-      <c r="E10" s="6" t="inlineStr"/>
-      <c r="F10" s="7" t="inlineStr">
+      <c r="E11" s="6" t="inlineStr"/>
+      <c r="F11" s="7" t="inlineStr">
         <is>
           <t>F-which-book.mp4</t>
         </is>
       </c>
-      <c r="G10" s="6" t="inlineStr"/>
-      <c r="H10" s="6" t="inlineStr">
+      <c r="G11" s="6" t="inlineStr"/>
+      <c r="H11" s="6" t="inlineStr">
         <is>
           <t>Which one would your kid pick? 1, 2, 3 or 4? 🦌🐻🛻🦄 Every page: one big picture to color + one easy sentence to read. Ages 3-6.
 1 Nico: https://www.amazon.com/dp/B0HLVTTK7T
@@ -1247,400 +1314,359 @@
 #kidsbooks #coloringbook #learningtoread #giftideasforkids</t>
         </is>
       </c>
-      <c r="I10" s="6" t="inlineStr">
+      <c r="I11" s="6" t="inlineStr">
         <is>
           <t>Comment 1, 2, 3 or 4! 👇</t>
         </is>
       </c>
-      <c r="J10" s="6" t="inlineStr">
+      <c r="J11" s="6" t="inlineStr">
         <is>
           <t>Reel. Then share to Story with a link sticker.</t>
         </is>
       </c>
     </row>
-    <row r="11" ht="155" customHeight="1">
-      <c r="A11" s="4" t="inlineStr">
+    <row r="12" ht="155" customHeight="1">
+      <c r="A12" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B11" s="5" t="inlineStr">
+      <c r="B12" s="5" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C11" s="5" t="inlineStr">
+      <c r="C12" s="5" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr">
+      <c r="D12" s="5" t="inlineStr">
         <is>
           <t>Rocco</t>
         </is>
       </c>
-      <c r="E11" s="6" t="inlineStr"/>
-      <c r="F11" s="7" t="inlineStr">
+      <c r="E12" s="6" t="inlineStr"/>
+      <c r="F12" s="7" t="inlineStr">
         <is>
           <t>C-rocco-spot-difference.mp4</t>
         </is>
       </c>
-      <c r="G11" s="6" t="inlineStr"/>
-      <c r="H11" s="6" t="inlineStr">
+      <c r="G12" s="6" t="inlineStr"/>
+      <c r="H12" s="6" t="inlineStr">
         <is>
           <t>Spot the difference: monster truck edition 🛻🔍 3 differences, 8 seconds. Can your kid beat the timer? Link in bio
 #spotthedifference #monstertruck #kidsgames #toddleractivities #puzzle</t>
         </is>
       </c>
-      <c r="I11" s="6" t="inlineStr">
+      <c r="I12" s="6" t="inlineStr">
         <is>
           <t>How many did you find? 1, 2 or 3? 👇</t>
         </is>
       </c>
-      <c r="J11" s="6" t="inlineStr">
+      <c r="J12" s="6" t="inlineStr">
         <is>
           <t>Already scheduled by Claude</t>
         </is>
       </c>
     </row>
-    <row r="12" ht="155" customHeight="1">
-      <c r="A12" s="4" t="inlineStr"/>
-      <c r="B12" s="8" t="inlineStr">
+    <row r="13" ht="155" customHeight="1">
+      <c r="A13" s="4" t="inlineStr"/>
+      <c r="B13" s="8" t="inlineStr">
         <is>
           <t>19:30</t>
         </is>
       </c>
-      <c r="C12" s="8" t="inlineStr">
+      <c r="C13" s="8" t="inlineStr">
         <is>
           <t>YouTube Shorts</t>
         </is>
       </c>
-      <c r="D12" s="8" t="inlineStr">
+      <c r="D13" s="8" t="inlineStr">
         <is>
           <t>Rocco</t>
         </is>
       </c>
-      <c r="E12" s="6" t="inlineStr"/>
-      <c r="F12" s="7" t="inlineStr">
+      <c r="E13" s="6" t="inlineStr"/>
+      <c r="F13" s="7" t="inlineStr">
         <is>
           <t>C-rocco-spot-difference.mp4</t>
         </is>
       </c>
-      <c r="G12" s="6" t="inlineStr">
+      <c r="G13" s="6" t="inlineStr">
         <is>
           <t>Spot 3 differences in 8 seconds! Monster truck edition 🛻 #shorts</t>
         </is>
       </c>
-      <c r="H12" s="6" t="inlineStr">
+      <c r="H13" s="6" t="inlineStr">
         <is>
           <t>Can your kid find all 3? From "Rocco the Little Monster Truck's Big Jump", a color &amp; read book for kids 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLZWLS5J
 #spotthedifference #monstertruck #kidsgames</t>
         </is>
       </c>
-      <c r="I12" s="6" t="inlineStr"/>
-      <c r="J12" s="6" t="inlineStr">
+      <c r="I13" s="6" t="inlineStr"/>
+      <c r="J13" s="6" t="inlineStr">
         <is>
           <t>Audience: NOT made for kids.</t>
         </is>
       </c>
     </row>
-    <row r="13" ht="120" customHeight="1">
-      <c r="A13" s="4" t="inlineStr"/>
-      <c r="B13" s="9" t="inlineStr">
+    <row r="14" ht="120" customHeight="1">
+      <c r="A14" s="4" t="inlineStr"/>
+      <c r="B14" s="9" t="inlineStr">
         <is>
           <t>20:00</t>
         </is>
       </c>
-      <c r="C13" s="9" t="inlineStr">
+      <c r="C14" s="9" t="inlineStr">
         <is>
           <t>Instagram + Facebook</t>
         </is>
       </c>
-      <c r="D13" s="9" t="inlineStr">
+      <c r="D14" s="9" t="inlineStr">
         <is>
           <t>Rocco</t>
         </is>
       </c>
-      <c r="E13" s="6" t="inlineStr"/>
-      <c r="F13" s="7" t="inlineStr">
+      <c r="E14" s="6" t="inlineStr"/>
+      <c r="F14" s="7" t="inlineStr">
         <is>
           <t>carousel-rocco-1.png</t>
         </is>
       </c>
-      <c r="G13" s="6" t="inlineStr"/>
-      <c r="H13" s="6" t="inlineStr">
-        <is>
-          <t>Spot 3 differences! 🛻🔍 Answers on slide 2 (no peeking). From Rocco's Big Jump: kids color every page AND read one easy sentence. Ages 3-6.
+      <c r="G14" s="6" t="inlineStr"/>
+      <c r="H14" s="6" t="inlineStr">
+        <is>
+          <t>Spot 3 differences! 🛻🔍 Answers on slide 2 (no peeking), then swipe to see a real page from the book. From Rocco's Big Jump: kids color every page AND read one easy sentence. Ages 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLZWLS5J (Instagram: link in bio)
 #spotthedifference #monstertruck #kidsactivities #toddleractivities</t>
         </is>
       </c>
-      <c r="I13" s="6" t="inlineStr">
+      <c r="I14" s="6" t="inlineStr">
         <is>
           <t>Found all 3? 👇</t>
         </is>
       </c>
-      <c r="J13" s="6" t="inlineStr">
-        <is>
-          <t>Photo post with 3 pictures in order: carousel-rocco-1, -2, -3.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="155" customHeight="1">
-      <c r="A14" s="4" t="inlineStr">
+      <c r="J14" s="6" t="inlineStr">
+        <is>
+          <t>Photo post with 5 pictures in order: carousel-rocco-1, -2, -3, -4, -5.</t>
+        </is>
+      </c>
+    </row>
+    <row r="15" ht="155" customHeight="1">
+      <c r="A15" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B14" s="5" t="inlineStr">
+      <c r="B15" s="5" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C14" s="5" t="inlineStr">
+      <c r="C15" s="5" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr">
+      <c r="D15" s="5" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="E14" s="6" t="inlineStr"/>
-      <c r="F14" s="7" t="inlineStr">
+      <c r="E15" s="6" t="inlineStr"/>
+      <c r="F15" s="7" t="inlineStr">
         <is>
           <t>D-nico-crayon-asmr.mp4</t>
         </is>
       </c>
-      <c r="G14" s="6" t="inlineStr"/>
-      <c r="H14" s="6" t="inlineStr">
+      <c r="G15" s="6" t="inlineStr"/>
+      <c r="H15" s="6" t="inlineStr">
         <is>
           <t>Crayon ASMR 🖍️ sound on. Coloring Nico the reindeer, Christmas edition ⛄ Link in bio
 #asmr #coloringasmr #satisfying #christmascoloring #coloringbook</t>
         </is>
       </c>
-      <c r="I14" s="6" t="inlineStr">
+      <c r="I15" s="6" t="inlineStr">
         <is>
           <t>What should we color next? 🖍️👇</t>
         </is>
       </c>
-      <c r="J14" s="6" t="inlineStr">
+      <c r="J15" s="6" t="inlineStr">
         <is>
           <t>Already scheduled by Claude</t>
         </is>
       </c>
     </row>
-    <row r="15" ht="155" customHeight="1">
-      <c r="A15" s="4" t="inlineStr"/>
-      <c r="B15" s="8" t="inlineStr">
+    <row r="16" ht="155" customHeight="1">
+      <c r="A16" s="4" t="inlineStr"/>
+      <c r="B16" s="8" t="inlineStr">
         <is>
           <t>20:30</t>
         </is>
       </c>
-      <c r="C15" s="8" t="inlineStr">
+      <c r="C16" s="8" t="inlineStr">
         <is>
           <t>YouTube Shorts</t>
         </is>
       </c>
-      <c r="D15" s="8" t="inlineStr">
+      <c r="D16" s="8" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="E15" s="6" t="inlineStr"/>
-      <c r="F15" s="7" t="inlineStr">
+      <c r="E16" s="6" t="inlineStr"/>
+      <c r="F16" s="7" t="inlineStr">
         <is>
           <t>A-nico-i-spy.mp4</t>
         </is>
       </c>
-      <c r="G15" s="6" t="inlineStr">
+      <c r="G16" s="6" t="inlineStr">
         <is>
           <t>I spy with my little eye... Christmas game for toddlers ⛄ #shorts</t>
         </is>
       </c>
-      <c r="H15" s="6" t="inlineStr">
+      <c r="H16" s="6" t="inlineStr">
         <is>
           <t>Play I spy with Nico the little reindeer! From "Nico the Little Reindeer's Snowy Day", a Christmas coloring book kids color AND read, ages 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLVTTK7T
 #ispy #christmascoloring #toddleractivities</t>
         </is>
       </c>
-      <c r="I15" s="6" t="inlineStr"/>
-      <c r="J15" s="6" t="inlineStr">
+      <c r="I16" s="6" t="inlineStr"/>
+      <c r="J16" s="6" t="inlineStr">
         <is>
           <t>Audience: NOT made for kids.</t>
         </is>
       </c>
     </row>
-    <row r="16" ht="155" customHeight="1">
-      <c r="A16" s="4" t="inlineStr"/>
-      <c r="B16" s="9" t="inlineStr">
+    <row r="17" ht="155" customHeight="1">
+      <c r="A17" s="4" t="inlineStr"/>
+      <c r="B17" s="9" t="inlineStr">
         <is>
           <t>21:00</t>
         </is>
       </c>
-      <c r="C16" s="9" t="inlineStr">
+      <c r="C17" s="9" t="inlineStr">
         <is>
           <t>Instagram + Facebook</t>
         </is>
       </c>
-      <c r="D16" s="9" t="inlineStr">
+      <c r="D17" s="9" t="inlineStr">
         <is>
           <t>Nico</t>
         </is>
       </c>
-      <c r="E16" s="6" t="inlineStr"/>
-      <c r="F16" s="7" t="inlineStr">
+      <c r="E17" s="6" t="inlineStr"/>
+      <c r="F17" s="7" t="inlineStr">
         <is>
           <t>A-nico-i-spy.mp4</t>
         </is>
       </c>
-      <c r="G16" s="6" t="inlineStr"/>
-      <c r="H16" s="6" t="inlineStr">
+      <c r="G17" s="6" t="inlineStr"/>
+      <c r="H17" s="6" t="inlineStr">
         <is>
           <t>I spy, with my little eye... 🦌 Play this with your toddler tonight! Nico's Snowy Day is a Christmas coloring book kids color AND read. Ages 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLVTTK7T (Instagram: link in bio)
 #ispy #toddleractivities #christmascoloring #stockingstuffer</t>
         </is>
       </c>
-      <c r="I16" s="6" t="inlineStr">
+      <c r="I17" s="6" t="inlineStr">
         <is>
           <t>Did they get all 3? 👇</t>
         </is>
       </c>
-      <c r="J16" s="6" t="inlineStr">
+      <c r="J17" s="6" t="inlineStr">
         <is>
           <t>Reel. Then share to Story with a link sticker.</t>
         </is>
       </c>
     </row>
-    <row r="17" ht="155" customHeight="1">
-      <c r="A17" s="4" t="inlineStr">
+    <row r="18" ht="155" customHeight="1">
+      <c r="A18" s="4" t="inlineStr">
         <is>
           <t>✓</t>
         </is>
       </c>
-      <c r="B17" s="5" t="inlineStr">
+      <c r="B18" s="5" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C17" s="5" t="inlineStr">
+      <c r="C18" s="5" t="inlineStr">
         <is>
           <t>TikTok</t>
         </is>
       </c>
-      <c r="D17" s="5" t="inlineStr">
+      <c r="D18" s="5" t="inlineStr">
         <is>
           <t>Benny</t>
         </is>
       </c>
-      <c r="E17" s="6" t="inlineStr"/>
-      <c r="F17" s="7" t="inlineStr">
+      <c r="E18" s="6" t="inlineStr"/>
+      <c r="F18" s="7" t="inlineStr">
         <is>
           <t>E-benny-i-spy.mp4</t>
         </is>
       </c>
-      <c r="G17" s="6" t="inlineStr"/>
-      <c r="H17" s="6" t="inlineStr">
+      <c r="G18" s="6" t="inlineStr"/>
+      <c r="H18" s="6" t="inlineStr">
         <is>
           <t>I spy for toddlers 🐻🦋 Find it before I count to 3! A cozy coloring book kids color AND read. Ages 3-6. Link in bio
 #ispy #toddleractivities #preschool #kidsgames #coloringbook</t>
         </is>
       </c>
-      <c r="I17" s="6" t="inlineStr">
+      <c r="I18" s="6" t="inlineStr">
         <is>
           <t>Did your toddler find Benny first? 🐻👇</t>
         </is>
       </c>
-      <c r="J17" s="6" t="inlineStr">
+      <c r="J18" s="6" t="inlineStr">
         <is>
           <t>Already scheduled by Claude</t>
         </is>
       </c>
     </row>
-    <row r="18" ht="155" customHeight="1">
-      <c r="A18" s="4" t="inlineStr"/>
-      <c r="B18" s="8" t="inlineStr">
+    <row r="19" ht="155" customHeight="1">
+      <c r="A19" s="4" t="inlineStr"/>
+      <c r="B19" s="8" t="inlineStr">
         <is>
           <t>21:30</t>
         </is>
       </c>
-      <c r="C18" s="8" t="inlineStr">
+      <c r="C19" s="8" t="inlineStr">
         <is>
           <t>YouTube Shorts</t>
         </is>
       </c>
-      <c r="D18" s="8" t="inlineStr">
+      <c r="D19" s="8" t="inlineStr">
         <is>
           <t>Benny</t>
         </is>
       </c>
-      <c r="E18" s="6" t="inlineStr"/>
-      <c r="F18" s="7" t="inlineStr">
+      <c r="E19" s="6" t="inlineStr"/>
+      <c r="F19" s="7" t="inlineStr">
         <is>
           <t>G-benny-crayon-asmr.mp4</t>
         </is>
       </c>
-      <c r="G18" s="6" t="inlineStr">
+      <c r="G19" s="6" t="inlineStr">
         <is>
           <t>Crayon ASMR: coloring Benny the bear and his kite 🖍️ (sound on) #shorts</t>
         </is>
       </c>
-      <c r="H18" s="6" t="inlineStr">
+      <c r="H19" s="6" t="inlineStr">
         <is>
           <t>Relaxing crayon sounds. From "Benny the Bear's Cozy Day", a color &amp; read book for kids 3-6.
 Get it on Amazon: https://www.amazon.com/dp/B0HLVSLXK7
 #asmr #coloring #satisfying</t>
         </is>
       </c>
-      <c r="I18" s="6" t="inlineStr"/>
-      <c r="J18" s="6" t="inlineStr">
-        <is>
-          <t>Audience: NOT made for kids.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19" ht="131.75" customHeight="1">
-      <c r="A19" s="4" t="inlineStr"/>
-      <c r="B19" s="10" t="inlineStr">
-        <is>
-          <t>any</t>
-        </is>
-      </c>
-      <c r="C19" s="10" t="inlineStr">
-        <is>
-          <t>Pinterest</t>
-        </is>
-      </c>
-      <c r="D19" s="10" t="inlineStr">
-        <is>
-          <t>Rocco</t>
-        </is>
-      </c>
-      <c r="E19" s="6" t="inlineStr"/>
-      <c r="F19" s="7" t="inlineStr">
-        <is>
-          <t>pin-1-rocco.png</t>
-        </is>
-      </c>
-      <c r="G19" s="6" t="inlineStr">
-        <is>
-          <t>Spot 3 Differences: Monster Truck Activity for Kids 3-6</t>
-        </is>
-      </c>
-      <c r="H19" s="6" t="inlineStr">
-        <is>
-          <t>A free spot the difference puzzle with Rocco the little monster truck. Screen-free activity for preschoolers. From a color &amp; read story book for ages 3-6.
-Destination link: https://www.amazon.com/dp/B0HLZWLS5J</t>
-        </is>
-      </c>
       <c r="I19" s="6" t="inlineStr"/>
       <c r="J19" s="6" t="inlineStr">
         <is>
-          <t>Board: Kids Activities. Link goes in the Destination field.</t>
+          <t>Audience: NOT made for kids.</t>
         </is>
       </c>
     </row>
@@ -1658,28 +1684,69 @@
       </c>
       <c r="D20" s="10" t="inlineStr">
         <is>
-          <t>Posy</t>
+          <t>Rocco</t>
         </is>
       </c>
       <c r="E20" s="6" t="inlineStr"/>
       <c r="F20" s="7" t="inlineStr">
         <is>
+          <t>pin-1-rocco.png</t>
+        </is>
+      </c>
+      <c r="G20" s="6" t="inlineStr">
+        <is>
+          <t>Spot 3 Differences: Monster Truck Activity for Kids 3-6</t>
+        </is>
+      </c>
+      <c r="H20" s="6" t="inlineStr">
+        <is>
+          <t>A free spot the difference puzzle with Rocco the little monster truck. Screen-free activity for preschoolers. From a color &amp; read story book for ages 3-6.
+Destination link: https://www.amazon.com/dp/B0HLZWLS5J</t>
+        </is>
+      </c>
+      <c r="I20" s="6" t="inlineStr"/>
+      <c r="J20" s="6" t="inlineStr">
+        <is>
+          <t>Board: Kids Activities. Link goes in the Destination field.</t>
+        </is>
+      </c>
+    </row>
+    <row r="21" ht="131.75" customHeight="1">
+      <c r="A21" s="4" t="inlineStr"/>
+      <c r="B21" s="10" t="inlineStr">
+        <is>
+          <t>any</t>
+        </is>
+      </c>
+      <c r="C21" s="10" t="inlineStr">
+        <is>
+          <t>Pinterest</t>
+        </is>
+      </c>
+      <c r="D21" s="10" t="inlineStr">
+        <is>
+          <t>Posy</t>
+        </is>
+      </c>
+      <c r="E21" s="6" t="inlineStr"/>
+      <c r="F21" s="7" t="inlineStr">
+        <is>
           <t>pin-2-posy.png</t>
         </is>
       </c>
-      <c r="G20" s="6" t="inlineStr">
+      <c r="G21" s="6" t="inlineStr">
         <is>
           <t>Learn Colors with a Unicorn: Coloring Page for Kids 3-6</t>
         </is>
       </c>
-      <c r="H20" s="6" t="inlineStr">
+      <c r="H21" s="6" t="inlineStr">
         <is>
           <t>Red strawberries! Posy the little unicorn teaches every color of the rainbow. A coloring book kids color AND read, ages 3-6.
 Destination link: https://www.amazon.com/dp/B0HLZF8NMX</t>
         </is>
       </c>
-      <c r="I20" s="6" t="inlineStr"/>
-      <c r="J20" s="6" t="inlineStr">
+      <c r="I21" s="6" t="inlineStr"/>
+      <c r="J21" s="6" t="inlineStr">
         <is>
           <t>Board: Learning Colors. Link goes in the Destination field.</t>
         </is>
@@ -1687,7 +1754,7 @@
     </row>
   </sheetData>
   <dataValidations count="1">
-    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
+    <dataValidation sqref="A5 A6 A7 A8 A9 A10 A11 A12 A13 A14 A15 A16 A17 A18 A19 A20 A21" showDropDown="0" showInputMessage="0" showErrorMessage="0" allowBlank="1" type="list">
       <formula1>"✓"</formula1>
     </dataValidation>
   </dataValidations>
@@ -1708,8 +1775,9 @@
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F18" r:id="rId14"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F19" r:id="rId15"/>
     <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F20" r:id="rId16"/>
+    <hyperlink xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" ref="F21" r:id="rId17"/>
   </hyperlinks>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
-  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId17"/>
+  <drawing xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="rId18"/>
 </worksheet>
 </file>
</xml_diff>